<commit_message>
Catálogo: RTI-024 só na porta de acesso privilegiado e notas de versão e de uso corrigidas
A aba Triagem listava a RTI-024 também na porta de mobilidade e e-mail (135 entradas para 134 riscos); no questionário
aplicado ela está só em acesso privilegiado. A aba Controle de versão passa a dizer que 98% dos riscos da v1 (131 de
134) caíam em cinco combinações e que os 118 ajustes reduziram o grau; a aba Como usar esclarece que, no instrumento,
probabilidade e impacto ficam fixos para preservar a comparação entre órgãos.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-riscos-ti-cidades-inteligentes.xlsx
+++ b/catalogo/catalogo-riscos-ti-cidades-inteligentes.xlsx
@@ -14926,7 +14926,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Recalibrados risco a risco. Na v1, 91% das linhas caíam em 5 combinações e tudo resultava em Alto ou Extremo, o que anulava a priorização. Trilha completa na aba 'Calibração P x I'.</t>
+          <t>Recalibrados risco a risco. Na v1, 98% das linhas (131 de 134) caíam em 5 combinações e 87 resultavam em Extremo, o que anulava a priorização; os 118 riscos alterados tiveram o grau reduzido. Trilha completa na aba 'Calibração P x I'.</t>
         </is>
       </c>
     </row>
@@ -21793,11 +21793,11 @@
         </is>
       </c>
       <c r="H18" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>RTI-083, RTI-085, RTI-024</t>
+          <t>RTI-083, RTI-085</t>
         </is>
       </c>
     </row>
@@ -22039,6 +22039,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="B26" s="11" t="inlineStr">
         <is>
@@ -32970,7 +32971,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Os valores de probabilidade e impacto são sugestões de partida da base de conhecimento; não substituem a avaliação no contexto real do órgão.</t>
+          <t>Os valores de probabilidade e impacto são sugestões de partida da base de conhecimento; não substituem a avaliação no contexto real do órgão. No instrumento de maturidade, P e I ficam fixos para preservar a comparação entre órgãos; recalibrá-los localmente serve ao uso da base fora do instrumento e torna os índices não comparáveis.</t>
         </is>
       </c>
     </row>

</xml_diff>